<commit_message>
added lunch deduction and aggregate functions
</commit_message>
<xml_diff>
--- a/data/becoSkillList.xlsx
+++ b/data/becoSkillList.xlsx
@@ -7,7 +7,9 @@
     <workbookView windowWidth="21267" windowHeight="8019"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="skill_list" sheetId="1" r:id="rId1"/>
+    <sheet name="designation_list" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -27,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="75">
   <si>
     <t>NAME</t>
   </si>
@@ -194,7 +196,7 @@
     <t>RW0723808557</t>
   </si>
   <si>
-    <t xml:space="preserve">ASHOK ROY </t>
+    <t>ASHOK ROY</t>
   </si>
   <si>
     <t>RW0907097796</t>
@@ -203,37 +205,55 @@
     <t>Medium</t>
   </si>
   <si>
-    <t xml:space="preserve">B N MAHAPATRO </t>
+    <t>B N MAHAPATRO</t>
   </si>
   <si>
     <t>RW1103006020</t>
   </si>
   <si>
+    <t>BASUDEO</t>
+  </si>
+  <si>
+    <t>RW0204008111</t>
+  </si>
+  <si>
+    <t>CHITRANJAN</t>
+  </si>
+  <si>
+    <t>RW1110162302</t>
+  </si>
+  <si>
+    <t>KARAN KUMAR</t>
+  </si>
+  <si>
+    <t>RW1223956402</t>
+  </si>
+  <si>
+    <t>V RAJA RAO</t>
+  </si>
+  <si>
+    <t>RW0611151520</t>
+  </si>
+  <si>
     <t>BALWINDER SINGH</t>
   </si>
   <si>
-    <t>BASUDEO</t>
-  </si>
-  <si>
-    <t>RW0204008111</t>
-  </si>
-  <si>
-    <t>CHITRANJAN</t>
-  </si>
-  <si>
-    <t>RW1110162302</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KARAN KUMAR </t>
-  </si>
-  <si>
-    <t>RW1223956402</t>
-  </si>
-  <si>
-    <t xml:space="preserve">V RAJA RAO </t>
-  </si>
-  <si>
-    <t>RW0611151520</t>
+    <t>Safety Pass No</t>
+  </si>
+  <si>
+    <t>Designation</t>
+  </si>
+  <si>
+    <t>Driver</t>
+  </si>
+  <si>
+    <t>Shift</t>
+  </si>
+  <si>
+    <t>Shift Start</t>
+  </si>
+  <si>
+    <t>Shift End</t>
   </si>
 </sst>
 </file>
@@ -255,18 +275,17 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="14"/>
       <color theme="0"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Consolas"/>
+      <charset val="134"/>
     </font>
     <font>
       <b/>
@@ -274,7 +293,6 @@
       <color theme="0"/>
       <name val="Calibri"/>
       <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -436,7 +454,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="37">
+  <fills count="42">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -445,26 +463,56 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="8" tint="-0.5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="9" tint="-0.5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF8CBAD"/>
+        <fgColor theme="4" tint="0.8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.8"/>
         <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.8"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
@@ -929,7 +977,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="12" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="12" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -953,16 +1001,16 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="16" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="13" borderId="16" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="13" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="14" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -971,129 +1019,146 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="19" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1637,374 +1702,374 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr defaultColWidth="8.79279279279279" defaultRowHeight="14.4" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="32.7117117117117" style="1" customWidth="1"/>
-    <col min="2" max="2" width="19.4504504504505" style="1" customWidth="1"/>
-    <col min="3" max="3" width="15" style="1" customWidth="1"/>
+    <col min="1" max="1" width="32.7117117117117" style="4" customWidth="1"/>
+    <col min="2" max="2" width="19.4504504504505" style="4" customWidth="1"/>
+    <col min="3" max="3" width="15" style="4" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="19.05" spans="1:3">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="7" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" ht="16.8" spans="1:3">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="10" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="3" ht="16.8" spans="1:3">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="10" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="4" ht="16.8" spans="1:3">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="10" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="5" ht="16.8" spans="1:3">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="10" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="6" ht="16.8" spans="1:3">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="10" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="7" ht="16.8" spans="1:3">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="10" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="8" ht="16.8" spans="1:3">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="10" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="9" ht="16.8" spans="1:3">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="10" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="10" ht="16.8" spans="1:3">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="10" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="11" ht="16.8" spans="1:3">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="10" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="12" ht="16.8" spans="1:3">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="B12" s="11" t="s">
+      <c r="B12" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="10" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="13" ht="16.8" spans="1:3">
-      <c r="A13" s="12" t="s">
+      <c r="A13" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="C13" s="10" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="14" ht="16.8" spans="1:3">
-      <c r="A14" s="12" t="s">
+      <c r="A14" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="B14" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="C14" s="10" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="15" ht="16.8" spans="1:3">
-      <c r="A15" s="12" t="s">
+      <c r="A15" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="C15" s="10" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="16" ht="16.8" spans="1:3">
-      <c r="A16" s="13" t="s">
+      <c r="A16" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="B16" s="8" t="s">
+      <c r="B16" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="C16" s="17" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="17" ht="16.8" spans="1:3">
-      <c r="A17" s="13" t="s">
+      <c r="A17" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="B17" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="C17" s="17" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="18" ht="16.8" spans="1:3">
-      <c r="A18" s="13" t="s">
+      <c r="A18" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="B18" s="8" t="s">
+      <c r="B18" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="C18" s="17" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="19" ht="16.8" spans="1:3">
-      <c r="A19" s="13" t="s">
+      <c r="A19" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="B19" s="8" t="s">
+      <c r="B19" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="C19" s="17" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="20" ht="16.8" spans="1:3">
-      <c r="A20" s="14" t="s">
+      <c r="A20" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="B20" s="8" t="s">
+      <c r="B20" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="C20" s="7" t="s">
+      <c r="C20" s="17" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="21" ht="16.8" spans="1:3">
-      <c r="A21" s="13" t="s">
+      <c r="A21" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="B21" s="8" t="s">
+      <c r="B21" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="C21" s="7" t="s">
+      <c r="C21" s="17" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="22" ht="16.8" spans="1:3">
-      <c r="A22" s="15" t="s">
+      <c r="A22" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="B22" s="8" t="s">
+      <c r="B22" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="C22" s="7" t="s">
+      <c r="C22" s="17" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="23" ht="16.8" spans="1:3">
-      <c r="A23" s="16" t="s">
+      <c r="A23" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="B23" s="8" t="s">
+      <c r="B23" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="C23" s="7" t="s">
+      <c r="C23" s="17" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="24" ht="16.8" spans="1:3">
-      <c r="A24" s="17" t="s">
+      <c r="A24" s="21" t="s">
         <v>49</v>
       </c>
-      <c r="B24" s="8" t="s">
+      <c r="B24" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="C24" s="7" t="s">
+      <c r="C24" s="17" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="25" ht="16.8" spans="1:3">
-      <c r="A25" s="17" t="s">
+      <c r="A25" s="21" t="s">
         <v>51</v>
       </c>
-      <c r="B25" s="8" t="s">
+      <c r="B25" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="C25" s="7" t="s">
+      <c r="C25" s="17" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="26" ht="16.8" spans="1:3">
-      <c r="A26" s="17" t="s">
+      <c r="A26" s="21" t="s">
         <v>53</v>
       </c>
-      <c r="B26" s="6" t="s">
+      <c r="B26" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="C26" s="7" t="s">
+      <c r="C26" s="17" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="27" ht="16.8" spans="1:3">
-      <c r="A27" s="18" t="s">
+      <c r="A27" s="22" t="s">
         <v>55</v>
       </c>
-      <c r="B27" s="8" t="s">
+      <c r="B27" s="23" t="s">
         <v>56</v>
       </c>
-      <c r="C27" s="7" t="s">
+      <c r="C27" s="24" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="28" ht="16.8" spans="1:3">
-      <c r="A28" s="19" t="s">
+      <c r="A28" s="25" t="s">
         <v>58</v>
       </c>
-      <c r="B28" s="8" t="s">
+      <c r="B28" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="C28" s="7" t="s">
+      <c r="C28" s="24" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="29" ht="16.8" spans="1:3">
-      <c r="A29" s="19" t="s">
+      <c r="A29" s="25" t="s">
         <v>60</v>
       </c>
-      <c r="B29" s="20">
+      <c r="B29" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="C29" s="24" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="30" ht="16.8" spans="1:3">
+      <c r="A30" s="25" t="s">
+        <v>62</v>
+      </c>
+      <c r="B30" s="23" t="s">
+        <v>63</v>
+      </c>
+      <c r="C30" s="24" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="31" ht="16.8" spans="1:3">
+      <c r="A31" s="26" t="s">
+        <v>64</v>
+      </c>
+      <c r="B31" s="23" t="s">
+        <v>65</v>
+      </c>
+      <c r="C31" s="24" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="32" ht="16.05" spans="1:3">
+      <c r="A32" s="26" t="s">
+        <v>66</v>
+      </c>
+      <c r="B32" s="27" t="s">
+        <v>67</v>
+      </c>
+      <c r="C32" s="24" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="34" ht="16.05" spans="1:3">
+      <c r="A34" s="25" t="s">
+        <v>68</v>
+      </c>
+      <c r="B34" s="28">
         <v>0</v>
       </c>
-      <c r="C29" s="7" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="30" ht="16.8" spans="1:3">
-      <c r="A30" s="19" t="s">
-        <v>61</v>
-      </c>
-      <c r="B30" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="C30" s="7" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="31" ht="16.8" spans="1:3">
-      <c r="A31" s="19" t="s">
-        <v>63</v>
-      </c>
-      <c r="B31" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="C31" s="7" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="32" ht="16.8" spans="1:3">
-      <c r="A32" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="B32" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="C32" s="7" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="33" ht="16.05" spans="1:3">
-      <c r="A33" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="B33" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="C33" s="7" t="s">
+      <c r="C34" s="24" t="s">
         <v>57</v>
       </c>
     </row>
@@ -2018,4 +2083,99 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultColWidth="8.79279279279279" defaultRowHeight="14.4" outlineLevelRow="6" outlineLevelCol="1"/>
+  <cols>
+    <col min="1" max="1" width="17.8558558558559" customWidth="1"/>
+    <col min="2" max="2" width="14.5585585585586" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="18.25" spans="1:2">
+      <c r="A1" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr defaultColWidth="8.79279279279279" defaultRowHeight="14.4" outlineLevelCol="2"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
 </file>
</xml_diff>